<commit_message>
Release 1.2.8 with dependency-aware manifest exports
</commit_message>
<xml_diff>
--- a/tools/manifest-excel/tbpedia-manifests.xlsx
+++ b/tools/manifest-excel/tbpedia-manifests.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zh-tw-reading-standard-V1" sheetId="1" r:id="Rb8aed9ba0e1f4f9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zh-tw-reading-advanced-V1" sheetId="2" r:id="Re2a7edc03b3846a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zh-tw-notes-essential-V1" sheetId="3" r:id="R32de1e69c4084467"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zhtw-notes-expanded-V1" sheetId="4" r:id="R09958831ce67421e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zhtw-notes-essential-V1" sheetId="5" r:id="R815c3ba255d14e21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zhtw-specialisation-ai-V1" sheetId="6" r:id="R7ad7343397984425"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zhtw-special-propagation-V1" sheetId="7" r:id="R975ba4cf4a814e54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zhtw-special-seclusion-V1" sheetId="8" r:id="R42a678df77e84d7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zh-tw-reading-standard-V1" sheetId="1" r:id="R1c1835b398464da2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zh-tw-reading-advanced-V1" sheetId="2" r:id="Rc65cca42309b44d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zh-tw-notes-essential-V1" sheetId="3" r:id="R0f3c806107764e33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zhtw-notes-expanded-V1" sheetId="4" r:id="Rd4d05fcd4fb04524"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zhtw-notes-essential-V1" sheetId="5" r:id="R769649d67448448f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zhtw-specialisation-ai-V1" sheetId="6" r:id="Rb2999c7a8bdd42a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zhtw-special-propagation-V1" sheetId="7" r:id="Ra1617de9268144f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zhtw-special-seclusion-V1" sheetId="8" r:id="R41a3add124cb43d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +47,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -64,6 +64,11 @@
         <x:fgColor rgb="FFFFF7DB"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -77,7 +82,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="11">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -100,6 +105,12 @@
     </x:xf>
     <x:xf numFmtId="201" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -582,7 +593,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D17" s="2" t="str">
-        <x:v>Capital C: collection version</x:v>
+        <x:v>Release manifest version (V1); tbpedia holds the identity</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -590,7 +601,7 @@
         <x:v>/minimumPluginVersion</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>1.1.0</x:v>
+        <x:v>1.2.0</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>string</x:v>
@@ -1100,6 +1111,34 @@
         <x:v>integer</x:v>
       </x:c>
       <x:c r="D59" s="2" t="str"/>
+    </x:row>
+    <x:row r="60" ht="30" customHeight="1">
+      <x:c r="A60" s="2" t="str">
+        <x:v>/releases/0/dependsOn</x:v>
+      </x:c>
+      <x:c r="B60" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C60" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D60" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="30" customHeight="1">
+      <x:c r="A61" s="2" t="str">
+        <x:v>/releases/1/dependsOn</x:v>
+      </x:c>
+      <x:c r="B61" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C61" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D61" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -1109,7 +1148,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9831eb452fe4010"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04494df9926e4545"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1301,7 +1340,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D17" s="2" t="str">
-        <x:v>Capital C: collection version</x:v>
+        <x:v>Release manifest version (V1); tbpedia holds the identity</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -1309,7 +1348,7 @@
         <x:v>/minimumPluginVersion</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>1.1.0</x:v>
+        <x:v>1.2.0</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>string</x:v>
@@ -1733,6 +1772,20 @@
         <x:v>integer</x:v>
       </x:c>
       <x:c r="D52" s="2" t="str"/>
+    </x:row>
+    <x:row r="53" ht="30" customHeight="1">
+      <x:c r="A53" s="2" t="str">
+        <x:v>/releases/0/dependsOn</x:v>
+      </x:c>
+      <x:c r="B53" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C53" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D53" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -1742,7 +1795,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a17d04e85e64f2c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rced2f6ff414342ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1934,7 +1987,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D17" s="2" t="str">
-        <x:v>Capital C: collection version</x:v>
+        <x:v>Release manifest version (V1); tbpedia holds the identity</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -1942,7 +1995,7 @@
         <x:v>/minimumPluginVersion</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>1.1.0</x:v>
+        <x:v>1.2.0</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>string</x:v>
@@ -2452,6 +2505,34 @@
         <x:v>integer</x:v>
       </x:c>
       <x:c r="D59" s="2" t="str"/>
+    </x:row>
+    <x:row r="60" ht="30" customHeight="1">
+      <x:c r="A60" s="2" t="str">
+        <x:v>/releases/0/dependsOn</x:v>
+      </x:c>
+      <x:c r="B60" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C60" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D60" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="30" customHeight="1">
+      <x:c r="A61" s="2" t="str">
+        <x:v>/releases/1/dependsOn</x:v>
+      </x:c>
+      <x:c r="B61" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C61" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D61" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -2461,7 +2542,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R672e8575a437461a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R003175aa8f0d42f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2653,7 +2734,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D17" s="2" t="str">
-        <x:v>Capital C: collection version</x:v>
+        <x:v>Release manifest version (V1); tbpedia holds the identity</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -2661,7 +2742,7 @@
         <x:v>/minimumPluginVersion</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>1.1.0</x:v>
+        <x:v>1.2.0</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>string</x:v>
@@ -3171,6 +3252,34 @@
         <x:v>integer</x:v>
       </x:c>
       <x:c r="D59" s="2" t="str"/>
+    </x:row>
+    <x:row r="60" ht="30" customHeight="1">
+      <x:c r="A60" s="2" t="str">
+        <x:v>/releases/0/dependsOn</x:v>
+      </x:c>
+      <x:c r="B60" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C60" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D60" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="30" customHeight="1">
+      <x:c r="A61" s="2" t="str">
+        <x:v>/releases/1/dependsOn</x:v>
+      </x:c>
+      <x:c r="B61" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C61" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D61" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -3180,7 +3289,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd6f8e23e00d4885"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra44746c26880444b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3372,7 +3481,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D17" s="2" t="str">
-        <x:v>Capital C: collection version</x:v>
+        <x:v>Release manifest version (V1); tbpedia holds the identity</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -3380,7 +3489,7 @@
         <x:v>/minimumPluginVersion</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>1.1.0</x:v>
+        <x:v>1.2.0</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>string</x:v>
@@ -3890,6 +3999,34 @@
         <x:v>integer</x:v>
       </x:c>
       <x:c r="D59" s="2" t="str"/>
+    </x:row>
+    <x:row r="60" ht="30" customHeight="1">
+      <x:c r="A60" s="2" t="str">
+        <x:v>/releases/0/dependsOn</x:v>
+      </x:c>
+      <x:c r="B60" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C60" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D60" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="30" customHeight="1">
+      <x:c r="A61" s="2" t="str">
+        <x:v>/releases/1/dependsOn</x:v>
+      </x:c>
+      <x:c r="B61" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C61" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D61" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -3899,7 +4036,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra16865aa30c14320"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3921956b3544453e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4091,7 +4228,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D17" s="2" t="str">
-        <x:v>Capital C: collection version</x:v>
+        <x:v>Release manifest version (V1); tbpedia holds the identity</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -4099,7 +4236,7 @@
         <x:v>/minimumPluginVersion</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>1.1.0</x:v>
+        <x:v>1.2.0</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>string</x:v>
@@ -4609,6 +4746,34 @@
         <x:v>integer</x:v>
       </x:c>
       <x:c r="D59" s="2" t="str"/>
+    </x:row>
+    <x:row r="60" ht="30" customHeight="1">
+      <x:c r="A60" s="2" t="str">
+        <x:v>/releases/0/dependsOn</x:v>
+      </x:c>
+      <x:c r="B60" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C60" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D60" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="30" customHeight="1">
+      <x:c r="A61" s="2" t="str">
+        <x:v>/releases/1/dependsOn</x:v>
+      </x:c>
+      <x:c r="B61" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C61" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D61" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -4618,7 +4783,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e5be226c3a944e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51f171ad931249b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4810,7 +4975,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D17" s="2" t="str">
-        <x:v>Capital C: collection version</x:v>
+        <x:v>Release manifest version (V1); tbpedia holds the identity</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -4818,7 +4983,7 @@
         <x:v>/minimumPluginVersion</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>1.1.0</x:v>
+        <x:v>1.2.0</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>string</x:v>
@@ -5328,6 +5493,34 @@
         <x:v>integer</x:v>
       </x:c>
       <x:c r="D59" s="2" t="str"/>
+    </x:row>
+    <x:row r="60" ht="30" customHeight="1">
+      <x:c r="A60" s="2" t="str">
+        <x:v>/releases/0/dependsOn</x:v>
+      </x:c>
+      <x:c r="B60" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C60" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D60" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="30" customHeight="1">
+      <x:c r="A61" s="2" t="str">
+        <x:v>/releases/1/dependsOn</x:v>
+      </x:c>
+      <x:c r="B61" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C61" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D61" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -5337,7 +5530,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37e54fb690244011"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7eca5f21ec449ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5529,7 +5722,7 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="D17" s="2" t="str">
-        <x:v>Capital C: collection version</x:v>
+        <x:v>Release manifest version (V1); tbpedia holds the identity</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -5537,7 +5730,7 @@
         <x:v>/minimumPluginVersion</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>1.1.0</x:v>
+        <x:v>1.2.0</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>string</x:v>
@@ -6047,6 +6240,34 @@
         <x:v>integer</x:v>
       </x:c>
       <x:c r="D59" s="2" t="str"/>
+    </x:row>
+    <x:row r="60" ht="30" customHeight="1">
+      <x:c r="A60" s="2" t="str">
+        <x:v>/releases/0/dependsOn</x:v>
+      </x:c>
+      <x:c r="B60" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C60" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D60" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="30" customHeight="1">
+      <x:c r="A61" s="2" t="str">
+        <x:v>/releases/1/dependsOn</x:v>
+      </x:c>
+      <x:c r="B61" s="9" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="C61" s="2" t="str">
+        <x:v>json</x:v>
+      </x:c>
+      <x:c r="D61" s="10" t="str">
+        <x:v>[] independent; list required earlier release IDs as JSON</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -6056,7 +6277,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c0071ed6a554cd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad0eaf08fca04efb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>